<commit_message>
add addional info on appendix
</commit_message>
<xml_diff>
--- a/appendix.xlsx
+++ b/appendix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\production_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82E866F0-2DE6-43AD-B0A0-71747BB56A68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AC7347C-9B48-48F8-BBED-8F87E770BC1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>КОЛИЧЕСТВО / QTY</t>
   </si>
@@ -61,6 +61,9 @@
   </si>
   <si>
     <t>ДОПЪЛНЕНИЕ КЪМ РАБОТНА ПОРЪЧКА № / APPENDIX TO ORDER NUMBER</t>
+  </si>
+  <si>
+    <t>ДОПЪЛНИТЕЛНА ИНФОРМАЦИЯ / ADDITIONAL INFORMAION</t>
   </si>
 </sst>
 </file>
@@ -84,17 +87,18 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="8"/>
-      <color theme="1"/>
-      <name val="Arial Unicode MS"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="3">
@@ -111,7 +115,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -208,46 +212,14 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
+      <top/>
+      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
         <color indexed="64"/>
       </left>
       <right style="thin">
@@ -263,7 +235,7 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="thin">
+      <right style="medium">
         <color indexed="64"/>
       </right>
       <top/>
@@ -273,14 +245,78 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="medium">
         <color indexed="64"/>
       </right>
       <top/>
-      <bottom style="thin">
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="double">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -289,47 +325,61 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -610,7 +660,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:K18"/>
+  <dimension ref="A2:L27"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
@@ -625,64 +675,64 @@
   <sheetData>
     <row r="2" spans="2:11" ht="15" thickBot="1"/>
     <row r="3" spans="2:11" ht="15" thickBot="1">
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="17"/>
-      <c r="D3" s="17"/>
-      <c r="E3" s="17"/>
-      <c r="F3" s="17"/>
-      <c r="G3" s="17"/>
-      <c r="H3" s="18"/>
-      <c r="I3" s="19"/>
-      <c r="J3" s="7"/>
-      <c r="K3" s="8"/>
-    </row>
-    <row r="4" spans="2:11" ht="19.8" customHeight="1">
-      <c r="B4" s="11" t="s">
+      <c r="C3" s="24"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="24"/>
+      <c r="F3" s="24"/>
+      <c r="G3" s="24"/>
+      <c r="H3" s="25"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="5"/>
+    </row>
+    <row r="4" spans="2:11" ht="19.8" customHeight="1" thickTop="1">
+      <c r="B4" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="E4" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10" t="s">
+      <c r="F4" s="8"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="I4" s="10" t="s">
+      <c r="I4" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="J4" s="10" t="s">
+      <c r="J4" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="K4" s="14" t="s">
+      <c r="K4" s="10" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="2:11" ht="24" customHeight="1">
-      <c r="B5" s="12"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="9" t="s">
+      <c r="B5" s="13"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="G5" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="H5" s="13"/>
-      <c r="I5" s="13"/>
-      <c r="J5" s="13"/>
-      <c r="K5" s="15"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="11"/>
     </row>
     <row r="6" spans="2:11">
       <c r="B6" s="2"/>
@@ -816,7 +866,7 @@
       <c r="J16" s="1"/>
       <c r="K16" s="3"/>
     </row>
-    <row r="17" spans="2:11">
+    <row r="17" spans="1:12">
       <c r="B17" s="2"/>
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
@@ -828,20 +878,105 @@
       <c r="J17" s="1"/>
       <c r="K17" s="3"/>
     </row>
-    <row r="18" spans="2:11" ht="15" thickBot="1">
-      <c r="B18" s="4"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
-      <c r="I18" s="5"/>
-      <c r="J18" s="5"/>
-      <c r="K18" s="6"/>
+    <row r="18" spans="1:12">
+      <c r="B18" s="2"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
+      <c r="J18" s="1"/>
+      <c r="K18" s="3"/>
+    </row>
+    <row r="19" spans="1:12">
+      <c r="A19" s="15"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+      <c r="G19" s="1"/>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
+      <c r="J19" s="1"/>
+      <c r="K19" s="3"/>
+    </row>
+    <row r="20" spans="1:12">
+      <c r="A20" s="15"/>
+      <c r="B20" s="2"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="1"/>
+      <c r="H20" s="1"/>
+      <c r="I20" s="1"/>
+      <c r="J20" s="1"/>
+      <c r="K20" s="3"/>
+    </row>
+    <row r="21" spans="1:12" ht="15" thickBot="1">
+      <c r="A21" s="15"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+      <c r="G21" s="1"/>
+      <c r="H21" s="1"/>
+      <c r="I21" s="1"/>
+      <c r="J21" s="1"/>
+      <c r="K21" s="3"/>
+    </row>
+    <row r="22" spans="1:12" ht="15" thickBot="1">
+      <c r="B22" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="C22" s="21"/>
+      <c r="D22" s="21"/>
+      <c r="E22" s="21"/>
+      <c r="F22" s="21"/>
+      <c r="G22" s="21"/>
+      <c r="H22" s="21"/>
+      <c r="I22" s="21"/>
+      <c r="J22" s="21"/>
+      <c r="K22" s="22"/>
+      <c r="L22" s="16"/>
+    </row>
+    <row r="23" spans="1:12">
+      <c r="A23" s="15"/>
+      <c r="B23" s="19"/>
+      <c r="K23" s="15"/>
+    </row>
+    <row r="24" spans="1:12">
+      <c r="A24" s="15"/>
+      <c r="K24" s="15"/>
+    </row>
+    <row r="25" spans="1:12">
+      <c r="A25" s="15"/>
+      <c r="K25" s="15"/>
+    </row>
+    <row r="26" spans="1:12">
+      <c r="A26" s="15"/>
+      <c r="K26" s="15"/>
+    </row>
+    <row r="27" spans="1:12" ht="15" thickBot="1">
+      <c r="A27" s="15"/>
+      <c r="B27" s="18"/>
+      <c r="C27" s="14"/>
+      <c r="D27" s="14"/>
+      <c r="E27" s="14"/>
+      <c r="F27" s="14"/>
+      <c r="G27" s="14"/>
+      <c r="H27" s="14"/>
+      <c r="I27" s="14"/>
+      <c r="J27" s="14"/>
+      <c r="K27" s="17"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
+    <mergeCell ref="B22:K22"/>
     <mergeCell ref="I4:I5"/>
     <mergeCell ref="J4:J5"/>
     <mergeCell ref="K4:K5"/>

</xml_diff>